<commit_message>
build(output): update generated financial Excel reports in output-app directory
- Regenerate Journal 2026.xlsx, BUKU BESAR 2026.xlsx, Neraca Lajur 2026.xlsx, and Neraca, RL, Arus Kas...xlsx.

- Add newly generated AUDIT_TRAIL.xlsx report file.
</commit_message>
<xml_diff>
--- a/output-app/Journal 2026.xlsx
+++ b/output-app/Journal 2026.xlsx
@@ -33,7 +33,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="9">
+  <numFmts count="10">
     <numFmt numFmtId="5" formatCode="&quot;$&quot;#,##0_);\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="7" formatCode="&quot;$&quot;#,##0.00_);\(&quot;$&quot;#,##0.00\)"/>
@@ -43,6 +43,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -406,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F121"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -618,22 +619,22 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>01 Jan 2026</v>
+        <v>02 Jan 2001</v>
       </c>
       <c r="B11" t="str">
-        <v>15.03.00</v>
+        <v>50.01.00</v>
       </c>
       <c r="C11" t="str">
-        <v>Persediaan Bahan Instalasi</v>
+        <v>Utang Usaha</v>
       </c>
       <c r="D11" t="str">
-        <v>Persediaan Bahan Instalasi (Asesoris &amp; Water Meter)</v>
-      </c>
-      <c r="E11">
-        <v>21696230000.277</v>
-      </c>
-      <c r="F11" t="str">
-        <v/>
+        <v>Voucher: Pembayaran Biaya Perpanjangan STNK Mobil Pick Up KH 1234 PU</v>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11">
+        <v>200000</v>
       </c>
     </row>
     <row r="12">
@@ -641,39 +642,39 @@
         <v/>
       </c>
       <c r="B12" t="str">
-        <v>71.01.00</v>
+        <v>97.06.20</v>
       </c>
       <c r="C12" t="str">
-        <v>Kekayaan Pemda Yang Dipisahkan</v>
+        <v>Pemeliharaan Kendaraan</v>
       </c>
       <c r="D12" t="str">
         <v/>
       </c>
-      <c r="E12" t="str">
-        <v/>
-      </c>
-      <c r="F12">
-        <v>21696230000.277</v>
+      <c r="E12">
+        <v>200000</v>
+      </c>
+      <c r="F12" t="str">
+        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>01 Jan 2026</v>
+        <v>02 Jan 2001</v>
       </c>
       <c r="B13" t="str">
-        <v>15.01.00</v>
+        <v>11.01.00</v>
       </c>
       <c r="C13" t="str">
-        <v>Persediaan Bahan Kimia</v>
+        <v>Kas</v>
       </c>
       <c r="D13" t="str">
-        <v>Persediaan Bahan Kimia &amp; BBM</v>
-      </c>
-      <c r="E13">
-        <v>644</v>
-      </c>
-      <c r="F13" t="str">
-        <v/>
+        <v>Bayar: Pembayaran Biaya Perpanjangan STNK Mobil Pick Up KH 1234 PU</v>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13">
+        <v>200000</v>
       </c>
     </row>
     <row r="14">
@@ -681,39 +682,39 @@
         <v/>
       </c>
       <c r="B14" t="str">
-        <v>71.01.00</v>
+        <v>50.01.00</v>
       </c>
       <c r="C14" t="str">
-        <v>Kekayaan Pemda Yang Dipisahkan</v>
+        <v>Utang Usaha</v>
       </c>
       <c r="D14" t="str">
         <v/>
       </c>
-      <c r="E14" t="str">
-        <v/>
-      </c>
-      <c r="F14">
-        <v>644</v>
+      <c r="E14">
+        <v>200000</v>
+      </c>
+      <c r="F14" t="str">
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>18 Mei 2026</v>
+        <v>02 Jan 2001</v>
       </c>
       <c r="B15" t="str">
-        <v>11.01.00</v>
+        <v>50.01.00</v>
       </c>
       <c r="C15" t="str">
-        <v>Kas</v>
+        <v>Utang Usaha</v>
       </c>
       <c r="D15" t="str">
-        <v>Penerimaan Rek Air (KOPERASI)</v>
-      </c>
-      <c r="E15">
-        <v>79000</v>
-      </c>
-      <c r="F15" t="str">
-        <v/>
+        <v>Voucher: Pembayaran Biaya Perpanjangan STNK Mobil Pick Up KH 1234 PU</v>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15">
+        <v>200000</v>
       </c>
     </row>
     <row r="16">
@@ -721,56 +722,56 @@
         <v/>
       </c>
       <c r="B16" t="str">
-        <v>13.01.00</v>
+        <v>97.06.20</v>
       </c>
       <c r="C16" t="str">
-        <v>Piutang Usaha</v>
+        <v>Pemeliharaan Kendaraan</v>
       </c>
       <c r="D16" t="str">
         <v/>
       </c>
-      <c r="E16" t="str">
-        <v/>
-      </c>
-      <c r="F16">
-        <v>44500</v>
+      <c r="E16">
+        <v>200000</v>
+      </c>
+      <c r="F16" t="str">
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v/>
+        <v>02 Jan 2001</v>
       </c>
       <c r="B17" t="str">
-        <v>81.02.50</v>
+        <v>11.01.00</v>
       </c>
       <c r="C17" t="str">
-        <v>Pendapatan Denda</v>
+        <v>Kas</v>
       </c>
       <c r="D17" t="str">
-        <v/>
+        <v>Bayar: Pembayaran Biaya Perpanjangan STNK Mobil Pick Up KH 1234 PU</v>
       </c>
       <c r="E17" t="str">
         <v/>
       </c>
       <c r="F17">
-        <v>34500</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>18 Mei 2026</v>
+        <v/>
       </c>
       <c r="B18" t="str">
-        <v>11.01.00</v>
+        <v>50.01.00</v>
       </c>
       <c r="C18" t="str">
-        <v>Kas</v>
+        <v>Utang Usaha</v>
       </c>
       <c r="D18" t="str">
-        <v>Penerimaan Rek Air (LOKET CABANG)</v>
+        <v/>
       </c>
       <c r="E18">
-        <v>361700</v>
+        <v>200000</v>
       </c>
       <c r="F18" t="str">
         <v/>
@@ -778,22 +779,22 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v/>
+        <v>02 Jan 2001</v>
       </c>
       <c r="B19" t="str">
-        <v>13.01.00</v>
+        <v>50.01.00</v>
       </c>
       <c r="C19" t="str">
-        <v>Piutang Usaha</v>
+        <v>Utang Usaha</v>
       </c>
       <c r="D19" t="str">
-        <v/>
+        <v>Voucher: Pembayaran Biaya Perpanjangan STNK Mobil Pick Up KH 1234 PU</v>
       </c>
       <c r="E19" t="str">
         <v/>
       </c>
       <c r="F19">
-        <v>180850</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="20">
@@ -801,24 +802,24 @@
         <v/>
       </c>
       <c r="B20" t="str">
-        <v>81.02.50</v>
+        <v>97.06.20</v>
       </c>
       <c r="C20" t="str">
-        <v>Pendapatan Denda</v>
+        <v>Pemeliharaan Kendaraan</v>
       </c>
       <c r="D20" t="str">
         <v/>
       </c>
-      <c r="E20" t="str">
-        <v/>
-      </c>
-      <c r="F20">
-        <v>180850</v>
+      <c r="E20">
+        <v>200000</v>
+      </c>
+      <c r="F20" t="str">
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>18 Mei 2026</v>
+        <v>02 Jan 2001</v>
       </c>
       <c r="B21" t="str">
         <v>11.01.00</v>
@@ -827,13 +828,13 @@
         <v>Kas</v>
       </c>
       <c r="D21" t="str">
-        <v>Penerimaan Rek Air (LOKET KANTOR)</v>
-      </c>
-      <c r="E21">
-        <v>302900</v>
-      </c>
-      <c r="F21" t="str">
-        <v/>
+        <v>Bayar: Pembayaran Biaya Perpanjangan STNK Mobil Pick Up KH 1234 PU</v>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21">
+        <v>200000</v>
       </c>
     </row>
     <row r="22">
@@ -841,79 +842,79 @@
         <v/>
       </c>
       <c r="B22" t="str">
-        <v>13.01.00</v>
+        <v>50.01.00</v>
       </c>
       <c r="C22" t="str">
-        <v>Piutang Usaha</v>
+        <v>Utang Usaha</v>
       </c>
       <c r="D22" t="str">
         <v/>
       </c>
-      <c r="E22" t="str">
-        <v/>
-      </c>
-      <c r="F22">
-        <v>156450</v>
+      <c r="E22">
+        <v>200000</v>
+      </c>
+      <c r="F22" t="str">
+        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v/>
+        <v>01 Jan 2026</v>
       </c>
       <c r="B23" t="str">
-        <v>81.02.50</v>
+        <v>15.03.00</v>
       </c>
       <c r="C23" t="str">
-        <v>Pendapatan Denda</v>
+        <v>Persediaan Bahan Instalasi</v>
       </c>
       <c r="D23" t="str">
-        <v/>
-      </c>
-      <c r="E23" t="str">
-        <v/>
-      </c>
-      <c r="F23">
-        <v>146450</v>
+        <v>Persediaan Bahan Instalasi (Asesoris &amp; Water Meter)</v>
+      </c>
+      <c r="E23">
+        <v>21696230000.277</v>
+      </c>
+      <c r="F23" t="str">
+        <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>18 Mei 2026</v>
+        <v/>
       </c>
       <c r="B24" t="str">
-        <v>11.01.00</v>
+        <v>71.01.00</v>
       </c>
       <c r="C24" t="str">
-        <v>Kas</v>
+        <v>Kekayaan Pemda Yang Dipisahkan</v>
       </c>
       <c r="D24" t="str">
-        <v>Penerimaan Rek Air (KOPERASI)</v>
-      </c>
-      <c r="E24">
-        <v>79000</v>
-      </c>
-      <c r="F24" t="str">
-        <v/>
+        <v/>
+      </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
+      <c r="F24">
+        <v>21696230000.277</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v/>
+        <v>01 Jan 2026</v>
       </c>
       <c r="B25" t="str">
-        <v>13.01.00</v>
+        <v>15.01.00</v>
       </c>
       <c r="C25" t="str">
-        <v>Piutang Usaha</v>
+        <v>Persediaan Bahan Kimia</v>
       </c>
       <c r="D25" t="str">
-        <v/>
-      </c>
-      <c r="E25" t="str">
-        <v/>
-      </c>
-      <c r="F25">
-        <v>44500</v>
+        <v>Persediaan Bahan Kimia &amp; BBM</v>
+      </c>
+      <c r="E25">
+        <v>644</v>
+      </c>
+      <c r="F25" t="str">
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -921,10 +922,10 @@
         <v/>
       </c>
       <c r="B26" t="str">
-        <v>81.02.50</v>
+        <v>71.01.00</v>
       </c>
       <c r="C26" t="str">
-        <v>Pendapatan Denda</v>
+        <v>Kekayaan Pemda Yang Dipisahkan</v>
       </c>
       <c r="D26" t="str">
         <v/>
@@ -933,24 +934,24 @@
         <v/>
       </c>
       <c r="F26">
-        <v>34500</v>
+        <v>644</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>18 Mei 2026</v>
+        <v>01 Jan 2026</v>
       </c>
       <c r="B27" t="str">
-        <v>11.01.00</v>
+        <v>15.03.00</v>
       </c>
       <c r="C27" t="str">
-        <v>Kas</v>
+        <v>Persediaan Bahan Instalasi</v>
       </c>
       <c r="D27" t="str">
-        <v>Penerimaan Rek Air (LOKET CABANG)</v>
+        <v>Persediaan Bahan Instalasi (Asesoris &amp; Water Meter)</v>
       </c>
       <c r="E27">
-        <v>361700</v>
+        <v>21696230000.277</v>
       </c>
       <c r="F27" t="str">
         <v/>
@@ -961,10 +962,10 @@
         <v/>
       </c>
       <c r="B28" t="str">
-        <v>13.01.00</v>
+        <v>71.01.00</v>
       </c>
       <c r="C28" t="str">
-        <v>Piutang Usaha</v>
+        <v>Kekayaan Pemda Yang Dipisahkan</v>
       </c>
       <c r="D28" t="str">
         <v/>
@@ -973,67 +974,67 @@
         <v/>
       </c>
       <c r="F28">
-        <v>180850</v>
+        <v>21696230000.277</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v/>
+        <v>01 Jan 2026</v>
       </c>
       <c r="B29" t="str">
-        <v>81.02.50</v>
+        <v>15.01.00</v>
       </c>
       <c r="C29" t="str">
-        <v>Pendapatan Denda</v>
+        <v>Persediaan Bahan Kimia</v>
       </c>
       <c r="D29" t="str">
-        <v/>
-      </c>
-      <c r="E29" t="str">
-        <v/>
-      </c>
-      <c r="F29">
-        <v>180850</v>
+        <v>Persediaan Bahan Kimia &amp; BBM</v>
+      </c>
+      <c r="E29">
+        <v>644</v>
+      </c>
+      <c r="F29" t="str">
+        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>18 Mei 2026</v>
+        <v/>
       </c>
       <c r="B30" t="str">
-        <v>11.01.00</v>
+        <v>71.01.00</v>
       </c>
       <c r="C30" t="str">
-        <v>Kas</v>
+        <v>Kekayaan Pemda Yang Dipisahkan</v>
       </c>
       <c r="D30" t="str">
-        <v>Penerimaan Rek Air (LOKET KANTOR)</v>
-      </c>
-      <c r="E30">
-        <v>302900</v>
-      </c>
-      <c r="F30" t="str">
-        <v/>
+        <v/>
+      </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
+      <c r="F30">
+        <v>644</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v/>
+        <v>01 Jan 2026</v>
       </c>
       <c r="B31" t="str">
-        <v>13.01.00</v>
+        <v>15.03.00</v>
       </c>
       <c r="C31" t="str">
-        <v>Piutang Usaha</v>
+        <v>Persediaan Bahan Instalasi</v>
       </c>
       <c r="D31" t="str">
-        <v/>
-      </c>
-      <c r="E31" t="str">
-        <v/>
-      </c>
-      <c r="F31">
-        <v>156450</v>
+        <v>Persediaan Bahan Instalasi (Asesoris &amp; Water Meter)</v>
+      </c>
+      <c r="E31">
+        <v>21696230000.277</v>
+      </c>
+      <c r="F31" t="str">
+        <v/>
       </c>
     </row>
     <row r="32">
@@ -1041,10 +1042,10 @@
         <v/>
       </c>
       <c r="B32" t="str">
-        <v>81.02.50</v>
+        <v>71.01.00</v>
       </c>
       <c r="C32" t="str">
-        <v>Pendapatan Denda</v>
+        <v>Kekayaan Pemda Yang Dipisahkan</v>
       </c>
       <c r="D32" t="str">
         <v/>
@@ -1053,24 +1054,24 @@
         <v/>
       </c>
       <c r="F32">
-        <v>146450</v>
+        <v>21696230000.277</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>18 Mei 2026</v>
+        <v>01 Jan 2026</v>
       </c>
       <c r="B33" t="str">
-        <v>11.01.00</v>
+        <v>15.01.00</v>
       </c>
       <c r="C33" t="str">
-        <v>Kas</v>
+        <v>Persediaan Bahan Kimia</v>
       </c>
       <c r="D33" t="str">
-        <v>Penerimaan Rek Air (KOPERASI)</v>
+        <v>Persediaan Bahan Kimia &amp; BBM</v>
       </c>
       <c r="E33">
-        <v>79000</v>
+        <v>644</v>
       </c>
       <c r="F33" t="str">
         <v/>
@@ -1081,10 +1082,10 @@
         <v/>
       </c>
       <c r="B34" t="str">
-        <v>13.01.00</v>
+        <v>71.01.00</v>
       </c>
       <c r="C34" t="str">
-        <v>Piutang Usaha</v>
+        <v>Kekayaan Pemda Yang Dipisahkan</v>
       </c>
       <c r="D34" t="str">
         <v/>
@@ -1093,67 +1094,67 @@
         <v/>
       </c>
       <c r="F34">
-        <v>44500</v>
+        <v>644</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v/>
+        <v>01 Jan 2026</v>
       </c>
       <c r="B35" t="str">
-        <v>81.02.50</v>
+        <v>15.03.00</v>
       </c>
       <c r="C35" t="str">
-        <v>Pendapatan Denda</v>
+        <v>Persediaan Bahan Instalasi</v>
       </c>
       <c r="D35" t="str">
-        <v/>
-      </c>
-      <c r="E35" t="str">
-        <v/>
-      </c>
-      <c r="F35">
-        <v>34500</v>
+        <v>Persediaan Bahan Instalasi (Asesoris &amp; Water Meter)</v>
+      </c>
+      <c r="E35">
+        <v>21696230000.277</v>
+      </c>
+      <c r="F35" t="str">
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>18 Mei 2026</v>
+        <v/>
       </c>
       <c r="B36" t="str">
-        <v>11.01.00</v>
+        <v>71.01.00</v>
       </c>
       <c r="C36" t="str">
-        <v>Kas</v>
+        <v>Kekayaan Pemda Yang Dipisahkan</v>
       </c>
       <c r="D36" t="str">
-        <v>Penerimaan Rek Air (LOKET CABANG)</v>
-      </c>
-      <c r="E36">
-        <v>361700</v>
-      </c>
-      <c r="F36" t="str">
-        <v/>
+        <v/>
+      </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
+      <c r="F36">
+        <v>21696230000.277</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v/>
+        <v>01 Jan 2026</v>
       </c>
       <c r="B37" t="str">
-        <v>13.01.00</v>
+        <v>15.01.00</v>
       </c>
       <c r="C37" t="str">
-        <v>Piutang Usaha</v>
+        <v>Persediaan Bahan Kimia</v>
       </c>
       <c r="D37" t="str">
-        <v/>
-      </c>
-      <c r="E37" t="str">
-        <v/>
-      </c>
-      <c r="F37">
-        <v>180850</v>
+        <v>Persediaan Bahan Kimia &amp; BBM</v>
+      </c>
+      <c r="E37">
+        <v>644</v>
+      </c>
+      <c r="F37" t="str">
+        <v/>
       </c>
     </row>
     <row r="38">
@@ -1161,10 +1162,10 @@
         <v/>
       </c>
       <c r="B38" t="str">
-        <v>81.02.50</v>
+        <v>71.01.00</v>
       </c>
       <c r="C38" t="str">
-        <v>Pendapatan Denda</v>
+        <v>Kekayaan Pemda Yang Dipisahkan</v>
       </c>
       <c r="D38" t="str">
         <v/>
@@ -1173,7 +1174,7 @@
         <v/>
       </c>
       <c r="F38">
-        <v>180850</v>
+        <v>644</v>
       </c>
     </row>
     <row r="39">
@@ -1187,10 +1188,10 @@
         <v>Kas</v>
       </c>
       <c r="D39" t="str">
-        <v>Penerimaan Rek Air (LOKET KANTOR)</v>
+        <v>Penerimaan Rek Air (KOPERASI)</v>
       </c>
       <c r="E39">
-        <v>302900</v>
+        <v>79000</v>
       </c>
       <c r="F39" t="str">
         <v/>
@@ -1213,7 +1214,7 @@
         <v/>
       </c>
       <c r="F40">
-        <v>156450</v>
+        <v>44500</v>
       </c>
     </row>
     <row r="41">
@@ -1233,24 +1234,24 @@
         <v/>
       </c>
       <c r="F41">
-        <v>146450</v>
+        <v>34500</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>21 Jan 2001</v>
+        <v>18 Mei 2026</v>
       </c>
       <c r="B42" t="str">
-        <v>15.01.00</v>
+        <v>11.01.00</v>
       </c>
       <c r="C42" t="str">
-        <v>Persediaan Bahan Kimia</v>
+        <v>Kas</v>
       </c>
       <c r="D42" t="str">
-        <v>Voucher: Pembayaran Belanja Bahan Habis Pakai Tawas dll</v>
+        <v>Penerimaan Rek Air (LOKET CABANG)</v>
       </c>
       <c r="E42">
-        <v>125000</v>
+        <v>361700</v>
       </c>
       <c r="F42" t="str">
         <v/>
@@ -1261,10 +1262,10 @@
         <v/>
       </c>
       <c r="B43" t="str">
-        <v>50.01.01</v>
+        <v>13.01.00</v>
       </c>
       <c r="C43" t="str">
-        <v>Utang Usaha - Bahan Kimia</v>
+        <v>Piutang Usaha</v>
       </c>
       <c r="D43" t="str">
         <v/>
@@ -1273,59 +1274,1579 @@
         <v/>
       </c>
       <c r="F43">
-        <v>125000</v>
+        <v>180850</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>21 Jan 2001</v>
+        <v/>
       </c>
       <c r="B44" t="str">
-        <v>11.01.00</v>
+        <v>81.02.50</v>
       </c>
       <c r="C44" t="str">
-        <v>Kas</v>
+        <v>Pendapatan Denda</v>
       </c>
       <c r="D44" t="str">
-        <v>Bayar: Pembayaran Belanja Bahan Habis Pakai Tawas dll</v>
+        <v/>
       </c>
       <c r="E44" t="str">
         <v/>
       </c>
       <c r="F44">
-        <v>125000</v>
+        <v>180850</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v/>
+        <v>18 Mei 2026</v>
       </c>
       <c r="B45" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Penerimaan Rek Air (LOKET KANTOR)</v>
+      </c>
+      <c r="E45">
+        <v>302900</v>
+      </c>
+      <c r="F45" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v/>
+      </c>
+      <c r="B46" t="str">
+        <v>13.01.00</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Piutang Usaha</v>
+      </c>
+      <c r="D46" t="str">
+        <v/>
+      </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
+      <c r="F46">
+        <v>156450</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v/>
+      </c>
+      <c r="B47" t="str">
+        <v>81.02.50</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Pendapatan Denda</v>
+      </c>
+      <c r="D47" t="str">
+        <v/>
+      </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
+      <c r="F47">
+        <v>146450</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>18 Mei 2026</v>
+      </c>
+      <c r="B48" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Penerimaan Rek Air (KOPERASI)</v>
+      </c>
+      <c r="E48">
+        <v>79000</v>
+      </c>
+      <c r="F48" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v/>
+      </c>
+      <c r="B49" t="str">
+        <v>13.01.00</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Piutang Usaha</v>
+      </c>
+      <c r="D49" t="str">
+        <v/>
+      </c>
+      <c r="E49" t="str">
+        <v/>
+      </c>
+      <c r="F49">
+        <v>44500</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v/>
+      </c>
+      <c r="B50" t="str">
+        <v>81.02.50</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Pendapatan Denda</v>
+      </c>
+      <c r="D50" t="str">
+        <v/>
+      </c>
+      <c r="E50" t="str">
+        <v/>
+      </c>
+      <c r="F50">
+        <v>34500</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>18 Mei 2026</v>
+      </c>
+      <c r="B51" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Penerimaan Rek Air (LOKET CABANG)</v>
+      </c>
+      <c r="E51">
+        <v>361700</v>
+      </c>
+      <c r="F51" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v/>
+      </c>
+      <c r="B52" t="str">
+        <v>13.01.00</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Piutang Usaha</v>
+      </c>
+      <c r="D52" t="str">
+        <v/>
+      </c>
+      <c r="E52" t="str">
+        <v/>
+      </c>
+      <c r="F52">
+        <v>180850</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v/>
+      </c>
+      <c r="B53" t="str">
+        <v>81.02.50</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Pendapatan Denda</v>
+      </c>
+      <c r="D53" t="str">
+        <v/>
+      </c>
+      <c r="E53" t="str">
+        <v/>
+      </c>
+      <c r="F53">
+        <v>180850</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>18 Mei 2026</v>
+      </c>
+      <c r="B54" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Penerimaan Rek Air (LOKET KANTOR)</v>
+      </c>
+      <c r="E54">
+        <v>302900</v>
+      </c>
+      <c r="F54" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v/>
+      </c>
+      <c r="B55" t="str">
+        <v>13.01.00</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Piutang Usaha</v>
+      </c>
+      <c r="D55" t="str">
+        <v/>
+      </c>
+      <c r="E55" t="str">
+        <v/>
+      </c>
+      <c r="F55">
+        <v>156450</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v/>
+      </c>
+      <c r="B56" t="str">
+        <v>81.02.50</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Pendapatan Denda</v>
+      </c>
+      <c r="D56" t="str">
+        <v/>
+      </c>
+      <c r="E56" t="str">
+        <v/>
+      </c>
+      <c r="F56">
+        <v>146450</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>18 Mei 2026</v>
+      </c>
+      <c r="B57" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Penerimaan Rek Air (KOPERASI)</v>
+      </c>
+      <c r="E57">
+        <v>79000</v>
+      </c>
+      <c r="F57" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v/>
+      </c>
+      <c r="B58" t="str">
+        <v>13.01.00</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Piutang Usaha</v>
+      </c>
+      <c r="D58" t="str">
+        <v/>
+      </c>
+      <c r="E58" t="str">
+        <v/>
+      </c>
+      <c r="F58">
+        <v>44500</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v/>
+      </c>
+      <c r="B59" t="str">
+        <v>81.02.50</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Pendapatan Denda</v>
+      </c>
+      <c r="D59" t="str">
+        <v/>
+      </c>
+      <c r="E59" t="str">
+        <v/>
+      </c>
+      <c r="F59">
+        <v>34500</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>18 Mei 2026</v>
+      </c>
+      <c r="B60" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Penerimaan Rek Air (LOKET CABANG)</v>
+      </c>
+      <c r="E60">
+        <v>361700</v>
+      </c>
+      <c r="F60" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v/>
+      </c>
+      <c r="B61" t="str">
+        <v>13.01.00</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Piutang Usaha</v>
+      </c>
+      <c r="D61" t="str">
+        <v/>
+      </c>
+      <c r="E61" t="str">
+        <v/>
+      </c>
+      <c r="F61">
+        <v>180850</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v/>
+      </c>
+      <c r="B62" t="str">
+        <v>81.02.50</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Pendapatan Denda</v>
+      </c>
+      <c r="D62" t="str">
+        <v/>
+      </c>
+      <c r="E62" t="str">
+        <v/>
+      </c>
+      <c r="F62">
+        <v>180850</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>18 Mei 2026</v>
+      </c>
+      <c r="B63" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Penerimaan Rek Air (LOKET KANTOR)</v>
+      </c>
+      <c r="E63">
+        <v>302900</v>
+      </c>
+      <c r="F63" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v/>
+      </c>
+      <c r="B64" t="str">
+        <v>13.01.00</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Piutang Usaha</v>
+      </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
+      <c r="E64" t="str">
+        <v/>
+      </c>
+      <c r="F64">
+        <v>156450</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v/>
+      </c>
+      <c r="B65" t="str">
+        <v>81.02.50</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Pendapatan Denda</v>
+      </c>
+      <c r="D65" t="str">
+        <v/>
+      </c>
+      <c r="E65" t="str">
+        <v/>
+      </c>
+      <c r="F65">
+        <v>146450</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>18 Mei 2026</v>
+      </c>
+      <c r="B66" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D66" t="str">
+        <v>Penerimaan Rek Air (KOPERASI)</v>
+      </c>
+      <c r="E66">
+        <v>79000</v>
+      </c>
+      <c r="F66" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v/>
+      </c>
+      <c r="B67" t="str">
+        <v>13.01.00</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Piutang Usaha</v>
+      </c>
+      <c r="D67" t="str">
+        <v/>
+      </c>
+      <c r="E67" t="str">
+        <v/>
+      </c>
+      <c r="F67">
+        <v>44500</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v/>
+      </c>
+      <c r="B68" t="str">
+        <v>81.02.50</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Pendapatan Denda</v>
+      </c>
+      <c r="D68" t="str">
+        <v/>
+      </c>
+      <c r="E68" t="str">
+        <v/>
+      </c>
+      <c r="F68">
+        <v>34500</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>18 Mei 2026</v>
+      </c>
+      <c r="B69" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Penerimaan Rek Air (LOKET CABANG)</v>
+      </c>
+      <c r="E69">
+        <v>361700</v>
+      </c>
+      <c r="F69" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v/>
+      </c>
+      <c r="B70" t="str">
+        <v>13.01.00</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Piutang Usaha</v>
+      </c>
+      <c r="D70" t="str">
+        <v/>
+      </c>
+      <c r="E70" t="str">
+        <v/>
+      </c>
+      <c r="F70">
+        <v>180850</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v/>
+      </c>
+      <c r="B71" t="str">
+        <v>81.02.50</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Pendapatan Denda</v>
+      </c>
+      <c r="D71" t="str">
+        <v/>
+      </c>
+      <c r="E71" t="str">
+        <v/>
+      </c>
+      <c r="F71">
+        <v>180850</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>18 Mei 2026</v>
+      </c>
+      <c r="B72" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D72" t="str">
+        <v>Penerimaan Rek Air (LOKET KANTOR)</v>
+      </c>
+      <c r="E72">
+        <v>302900</v>
+      </c>
+      <c r="F72" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v/>
+      </c>
+      <c r="B73" t="str">
+        <v>13.01.00</v>
+      </c>
+      <c r="C73" t="str">
+        <v>Piutang Usaha</v>
+      </c>
+      <c r="D73" t="str">
+        <v/>
+      </c>
+      <c r="E73" t="str">
+        <v/>
+      </c>
+      <c r="F73">
+        <v>156450</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v/>
+      </c>
+      <c r="B74" t="str">
+        <v>81.02.50</v>
+      </c>
+      <c r="C74" t="str">
+        <v>Pendapatan Denda</v>
+      </c>
+      <c r="D74" t="str">
+        <v/>
+      </c>
+      <c r="E74" t="str">
+        <v/>
+      </c>
+      <c r="F74">
+        <v>146450</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>18 Mei 2026</v>
+      </c>
+      <c r="B75" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C75" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D75" t="str">
+        <v>Penerimaan Rek Air (KOPERASI)</v>
+      </c>
+      <c r="E75">
+        <v>79000</v>
+      </c>
+      <c r="F75" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v/>
+      </c>
+      <c r="B76" t="str">
+        <v>13.01.00</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Piutang Usaha</v>
+      </c>
+      <c r="D76" t="str">
+        <v/>
+      </c>
+      <c r="E76" t="str">
+        <v/>
+      </c>
+      <c r="F76">
+        <v>44500</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v/>
+      </c>
+      <c r="B77" t="str">
+        <v>81.02.50</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Pendapatan Denda</v>
+      </c>
+      <c r="D77" t="str">
+        <v/>
+      </c>
+      <c r="E77" t="str">
+        <v/>
+      </c>
+      <c r="F77">
+        <v>34500</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>18 Mei 2026</v>
+      </c>
+      <c r="B78" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C78" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D78" t="str">
+        <v>Penerimaan Rek Air (LOKET CABANG)</v>
+      </c>
+      <c r="E78">
+        <v>361700</v>
+      </c>
+      <c r="F78" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v/>
+      </c>
+      <c r="B79" t="str">
+        <v>13.01.00</v>
+      </c>
+      <c r="C79" t="str">
+        <v>Piutang Usaha</v>
+      </c>
+      <c r="D79" t="str">
+        <v/>
+      </c>
+      <c r="E79" t="str">
+        <v/>
+      </c>
+      <c r="F79">
+        <v>180850</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v/>
+      </c>
+      <c r="B80" t="str">
+        <v>81.02.50</v>
+      </c>
+      <c r="C80" t="str">
+        <v>Pendapatan Denda</v>
+      </c>
+      <c r="D80" t="str">
+        <v/>
+      </c>
+      <c r="E80" t="str">
+        <v/>
+      </c>
+      <c r="F80">
+        <v>180850</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>18 Mei 2026</v>
+      </c>
+      <c r="B81" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C81" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D81" t="str">
+        <v>Penerimaan Rek Air (LOKET KANTOR)</v>
+      </c>
+      <c r="E81">
+        <v>302900</v>
+      </c>
+      <c r="F81" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v/>
+      </c>
+      <c r="B82" t="str">
+        <v>13.01.00</v>
+      </c>
+      <c r="C82" t="str">
+        <v>Piutang Usaha</v>
+      </c>
+      <c r="D82" t="str">
+        <v/>
+      </c>
+      <c r="E82" t="str">
+        <v/>
+      </c>
+      <c r="F82">
+        <v>156450</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v/>
+      </c>
+      <c r="B83" t="str">
+        <v>81.02.50</v>
+      </c>
+      <c r="C83" t="str">
+        <v>Pendapatan Denda</v>
+      </c>
+      <c r="D83" t="str">
+        <v/>
+      </c>
+      <c r="E83" t="str">
+        <v/>
+      </c>
+      <c r="F83">
+        <v>146450</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>18 Mei 2026</v>
+      </c>
+      <c r="B84" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C84" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D84" t="str">
+        <v>Penerimaan Rek Air (KOPERASI)</v>
+      </c>
+      <c r="E84">
+        <v>79000</v>
+      </c>
+      <c r="F84" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v/>
+      </c>
+      <c r="B85" t="str">
+        <v>13.01.00</v>
+      </c>
+      <c r="C85" t="str">
+        <v>Piutang Usaha</v>
+      </c>
+      <c r="D85" t="str">
+        <v/>
+      </c>
+      <c r="E85" t="str">
+        <v/>
+      </c>
+      <c r="F85">
+        <v>44500</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v/>
+      </c>
+      <c r="B86" t="str">
+        <v>81.02.50</v>
+      </c>
+      <c r="C86" t="str">
+        <v>Pendapatan Denda</v>
+      </c>
+      <c r="D86" t="str">
+        <v/>
+      </c>
+      <c r="E86" t="str">
+        <v/>
+      </c>
+      <c r="F86">
+        <v>34500</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>18 Mei 2026</v>
+      </c>
+      <c r="B87" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C87" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D87" t="str">
+        <v>Penerimaan Rek Air (LOKET CABANG)</v>
+      </c>
+      <c r="E87">
+        <v>361700</v>
+      </c>
+      <c r="F87" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v/>
+      </c>
+      <c r="B88" t="str">
+        <v>13.01.00</v>
+      </c>
+      <c r="C88" t="str">
+        <v>Piutang Usaha</v>
+      </c>
+      <c r="D88" t="str">
+        <v/>
+      </c>
+      <c r="E88" t="str">
+        <v/>
+      </c>
+      <c r="F88">
+        <v>180850</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v/>
+      </c>
+      <c r="B89" t="str">
+        <v>81.02.50</v>
+      </c>
+      <c r="C89" t="str">
+        <v>Pendapatan Denda</v>
+      </c>
+      <c r="D89" t="str">
+        <v/>
+      </c>
+      <c r="E89" t="str">
+        <v/>
+      </c>
+      <c r="F89">
+        <v>180850</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>18 Mei 2026</v>
+      </c>
+      <c r="B90" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C90" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D90" t="str">
+        <v>Penerimaan Rek Air (LOKET KANTOR)</v>
+      </c>
+      <c r="E90">
+        <v>302900</v>
+      </c>
+      <c r="F90" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v/>
+      </c>
+      <c r="B91" t="str">
+        <v>13.01.00</v>
+      </c>
+      <c r="C91" t="str">
+        <v>Piutang Usaha</v>
+      </c>
+      <c r="D91" t="str">
+        <v/>
+      </c>
+      <c r="E91" t="str">
+        <v/>
+      </c>
+      <c r="F91">
+        <v>156450</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v/>
+      </c>
+      <c r="B92" t="str">
+        <v>81.02.50</v>
+      </c>
+      <c r="C92" t="str">
+        <v>Pendapatan Denda</v>
+      </c>
+      <c r="D92" t="str">
+        <v/>
+      </c>
+      <c r="E92" t="str">
+        <v/>
+      </c>
+      <c r="F92">
+        <v>146450</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>18 Mei 2026</v>
+      </c>
+      <c r="B93" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C93" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D93" t="str">
+        <v>Penerimaan Rek Air (KOPERASI)</v>
+      </c>
+      <c r="E93">
+        <v>79000</v>
+      </c>
+      <c r="F93" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v/>
+      </c>
+      <c r="B94" t="str">
+        <v>13.01.00</v>
+      </c>
+      <c r="C94" t="str">
+        <v>Piutang Usaha</v>
+      </c>
+      <c r="D94" t="str">
+        <v/>
+      </c>
+      <c r="E94" t="str">
+        <v/>
+      </c>
+      <c r="F94">
+        <v>44500</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v/>
+      </c>
+      <c r="B95" t="str">
+        <v>81.02.50</v>
+      </c>
+      <c r="C95" t="str">
+        <v>Pendapatan Denda</v>
+      </c>
+      <c r="D95" t="str">
+        <v/>
+      </c>
+      <c r="E95" t="str">
+        <v/>
+      </c>
+      <c r="F95">
+        <v>34500</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>18 Mei 2026</v>
+      </c>
+      <c r="B96" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C96" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D96" t="str">
+        <v>Penerimaan Rek Air (LOKET CABANG)</v>
+      </c>
+      <c r="E96">
+        <v>361700</v>
+      </c>
+      <c r="F96" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v/>
+      </c>
+      <c r="B97" t="str">
+        <v>13.01.00</v>
+      </c>
+      <c r="C97" t="str">
+        <v>Piutang Usaha</v>
+      </c>
+      <c r="D97" t="str">
+        <v/>
+      </c>
+      <c r="E97" t="str">
+        <v/>
+      </c>
+      <c r="F97">
+        <v>180850</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v/>
+      </c>
+      <c r="B98" t="str">
+        <v>81.02.50</v>
+      </c>
+      <c r="C98" t="str">
+        <v>Pendapatan Denda</v>
+      </c>
+      <c r="D98" t="str">
+        <v/>
+      </c>
+      <c r="E98" t="str">
+        <v/>
+      </c>
+      <c r="F98">
+        <v>180850</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>18 Mei 2026</v>
+      </c>
+      <c r="B99" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C99" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D99" t="str">
+        <v>Penerimaan Rek Air (LOKET KANTOR)</v>
+      </c>
+      <c r="E99">
+        <v>302900</v>
+      </c>
+      <c r="F99" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v/>
+      </c>
+      <c r="B100" t="str">
+        <v>13.01.00</v>
+      </c>
+      <c r="C100" t="str">
+        <v>Piutang Usaha</v>
+      </c>
+      <c r="D100" t="str">
+        <v/>
+      </c>
+      <c r="E100" t="str">
+        <v/>
+      </c>
+      <c r="F100">
+        <v>156450</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v/>
+      </c>
+      <c r="B101" t="str">
+        <v>81.02.50</v>
+      </c>
+      <c r="C101" t="str">
+        <v>Pendapatan Denda</v>
+      </c>
+      <c r="D101" t="str">
+        <v/>
+      </c>
+      <c r="E101" t="str">
+        <v/>
+      </c>
+      <c r="F101">
+        <v>146450</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>24 Jul 2026</v>
+      </c>
+      <c r="B102" t="str">
+        <v>15.01.00</v>
+      </c>
+      <c r="C102" t="str">
+        <v>Persediaan Bahan Kimia</v>
+      </c>
+      <c r="D102" t="str">
+        <v>PEMBELIAN KAPORIT</v>
+      </c>
+      <c r="E102">
+        <v>100000</v>
+      </c>
+      <c r="F102">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v/>
+      </c>
+      <c r="B103" t="str">
+        <v>97.06.20</v>
+      </c>
+      <c r="C103" t="str">
+        <v>Pemeliharaan Kendaraan</v>
+      </c>
+      <c r="D103" t="str">
+        <v/>
+      </c>
+      <c r="E103" t="str">
+        <v/>
+      </c>
+      <c r="F103" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>24 Jul 2026</v>
+      </c>
+      <c r="B104" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C104" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D104" t="str">
+        <v>Tes Transaksi Terbaru Paling Atas</v>
+      </c>
+      <c r="E104">
+        <v>500000</v>
+      </c>
+      <c r="F104" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v/>
+      </c>
+      <c r="B105" t="str">
+        <v>81.01.10</v>
+      </c>
+      <c r="C105" t="str">
+        <v>Pendapatan Harga Air</v>
+      </c>
+      <c r="D105" t="str">
+        <v/>
+      </c>
+      <c r="E105" t="str">
+        <v/>
+      </c>
+      <c r="F105">
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>21 Jan 2001</v>
+      </c>
+      <c r="B106" t="str">
+        <v>15.01.00</v>
+      </c>
+      <c r="C106" t="str">
+        <v>Persediaan Bahan Kimia</v>
+      </c>
+      <c r="D106" t="str">
+        <v>Voucher: Pembayaran Belanja Bahan Habis Pakai Tawas dll</v>
+      </c>
+      <c r="E106">
+        <v>125000</v>
+      </c>
+      <c r="F106" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v/>
+      </c>
+      <c r="B107" t="str">
+        <v>50.01.01</v>
+      </c>
+      <c r="C107" t="str">
+        <v>Utang Usaha - Bahan Kimia</v>
+      </c>
+      <c r="D107" t="str">
+        <v/>
+      </c>
+      <c r="E107" t="str">
+        <v/>
+      </c>
+      <c r="F107">
+        <v>125000</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>21 Jan 2001</v>
+      </c>
+      <c r="B108" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C108" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D108" t="str">
+        <v>Bayar: Pembayaran Belanja Bahan Habis Pakai Tawas dll</v>
+      </c>
+      <c r="E108" t="str">
+        <v/>
+      </c>
+      <c r="F108">
+        <v>125000</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v/>
+      </c>
+      <c r="B109" t="str">
         <v>50.01.00</v>
       </c>
-      <c r="C45" t="str">
+      <c r="C109" t="str">
         <v>Utang Usaha</v>
       </c>
-      <c r="D45" t="str">
-        <v/>
-      </c>
-      <c r="E45">
+      <c r="D109" t="str">
+        <v/>
+      </c>
+      <c r="E109">
         <v>125000</v>
       </c>
-      <c r="F45" t="str">
+      <c r="F109" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>21 Jan 2001</v>
+      </c>
+      <c r="B110" t="str">
+        <v>15.01.00</v>
+      </c>
+      <c r="C110" t="str">
+        <v>Persediaan Bahan Kimia</v>
+      </c>
+      <c r="D110" t="str">
+        <v>Voucher: Pembayaran Belanja Bahan Habis Pakai Tawas dll</v>
+      </c>
+      <c r="E110">
+        <v>125000</v>
+      </c>
+      <c r="F110" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v/>
+      </c>
+      <c r="B111" t="str">
+        <v>50.01.01</v>
+      </c>
+      <c r="C111" t="str">
+        <v>Utang Usaha - Bahan Kimia</v>
+      </c>
+      <c r="D111" t="str">
+        <v/>
+      </c>
+      <c r="E111" t="str">
+        <v/>
+      </c>
+      <c r="F111">
+        <v>125000</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>21 Jan 2001</v>
+      </c>
+      <c r="B112" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C112" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D112" t="str">
+        <v>Bayar: Pembayaran Belanja Bahan Habis Pakai Tawas dll</v>
+      </c>
+      <c r="E112" t="str">
+        <v/>
+      </c>
+      <c r="F112">
+        <v>125000</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v/>
+      </c>
+      <c r="B113" t="str">
+        <v>50.01.00</v>
+      </c>
+      <c r="C113" t="str">
+        <v>Utang Usaha</v>
+      </c>
+      <c r="D113" t="str">
+        <v/>
+      </c>
+      <c r="E113">
+        <v>125000</v>
+      </c>
+      <c r="F113" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>21 Jan 2001</v>
+      </c>
+      <c r="B114" t="str">
+        <v>15.01.00</v>
+      </c>
+      <c r="C114" t="str">
+        <v>Persediaan Bahan Kimia</v>
+      </c>
+      <c r="D114" t="str">
+        <v>Voucher: Pembayaran Belanja Bahan Habis Pakai Tawas dll</v>
+      </c>
+      <c r="E114">
+        <v>125000</v>
+      </c>
+      <c r="F114" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v/>
+      </c>
+      <c r="B115" t="str">
+        <v>50.01.01</v>
+      </c>
+      <c r="C115" t="str">
+        <v>Utang Usaha - Bahan Kimia</v>
+      </c>
+      <c r="D115" t="str">
+        <v/>
+      </c>
+      <c r="E115" t="str">
+        <v/>
+      </c>
+      <c r="F115">
+        <v>125000</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>21 Jan 2001</v>
+      </c>
+      <c r="B116" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C116" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D116" t="str">
+        <v>Bayar: Pembayaran Belanja Bahan Habis Pakai Tawas dll</v>
+      </c>
+      <c r="E116" t="str">
+        <v/>
+      </c>
+      <c r="F116">
+        <v>125000</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v/>
+      </c>
+      <c r="B117" t="str">
+        <v>50.01.00</v>
+      </c>
+      <c r="C117" t="str">
+        <v>Utang Usaha</v>
+      </c>
+      <c r="D117" t="str">
+        <v/>
+      </c>
+      <c r="E117">
+        <v>125000</v>
+      </c>
+      <c r="F117" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>21 Jan 2001</v>
+      </c>
+      <c r="B118" t="str">
+        <v>15.01.00</v>
+      </c>
+      <c r="C118" t="str">
+        <v>Persediaan Bahan Kimia</v>
+      </c>
+      <c r="D118" t="str">
+        <v>Voucher: Pembayaran Belanja Bahan Habis Pakai Tawas dll</v>
+      </c>
+      <c r="E118">
+        <v>125000</v>
+      </c>
+      <c r="F118" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v/>
+      </c>
+      <c r="B119" t="str">
+        <v>50.01.01</v>
+      </c>
+      <c r="C119" t="str">
+        <v>Utang Usaha - Bahan Kimia</v>
+      </c>
+      <c r="D119" t="str">
+        <v/>
+      </c>
+      <c r="E119" t="str">
+        <v/>
+      </c>
+      <c r="F119">
+        <v>125000</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>21 Jan 2001</v>
+      </c>
+      <c r="B120" t="str">
+        <v>11.01.00</v>
+      </c>
+      <c r="C120" t="str">
+        <v>Kas</v>
+      </c>
+      <c r="D120" t="str">
+        <v>Bayar: Pembayaran Belanja Bahan Habis Pakai Tawas dll</v>
+      </c>
+      <c r="E120" t="str">
+        <v/>
+      </c>
+      <c r="F120">
+        <v>125000</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v/>
+      </c>
+      <c r="B121" t="str">
+        <v>50.01.00</v>
+      </c>
+      <c r="C121" t="str">
+        <v>Utang Usaha</v>
+      </c>
+      <c r="D121" t="str">
+        <v/>
+      </c>
+      <c r="E121">
+        <v>125000</v>
+      </c>
+      <c r="F121" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F45"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F121"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K14"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -1587,42 +3108,252 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v>02 Jan</v>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v>Voucher: Pembayaran Biaya Perpanjangan STNK Mobil Pick Up KH 1234 PU</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v>97.06.20</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Pemeliharaan Kendaraan</v>
+      </c>
+      <c r="H8">
+        <v>200000</v>
+      </c>
+      <c r="I8" t="str">
+        <v>50.01.00</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Utang Usaha</v>
+      </c>
+      <c r="K8">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>02 Jan</v>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
+        <v>Voucher: Pembayaran Biaya Perpanjangan STNK Mobil Pick Up KH 1234 PU</v>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v>97.06.20</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Pemeliharaan Kendaraan</v>
+      </c>
+      <c r="H9">
+        <v>200000</v>
+      </c>
+      <c r="I9" t="str">
+        <v>50.01.00</v>
+      </c>
+      <c r="J9" t="str">
+        <v>Utang Usaha</v>
+      </c>
+      <c r="K9">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>02 Jan</v>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v>Voucher: Pembayaran Biaya Perpanjangan STNK Mobil Pick Up KH 1234 PU</v>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v>97.06.20</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Pemeliharaan Kendaraan</v>
+      </c>
+      <c r="H10">
+        <v>200000</v>
+      </c>
+      <c r="I10" t="str">
+        <v>50.01.00</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Utang Usaha</v>
+      </c>
+      <c r="K10">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
         <v>21 Jan</v>
       </c>
-      <c r="B8" t="str">
-        <v/>
-      </c>
-      <c r="C8" t="str">
+      <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
         <v>Voucher: Pembayaran Belanja Bahan Habis Pakai Tawas dll</v>
       </c>
-      <c r="D8" t="str">
-        <v/>
-      </c>
-      <c r="E8" t="str">
-        <v/>
-      </c>
-      <c r="F8" t="str">
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
         <v>15.01.00</v>
       </c>
-      <c r="G8" t="str">
+      <c r="G11" t="str">
         <v>Persediaan Bahan Kimia</v>
       </c>
-      <c r="H8">
+      <c r="H11">
         <v>125000</v>
       </c>
-      <c r="I8" t="str">
+      <c r="I11" t="str">
         <v>50.01.01</v>
       </c>
-      <c r="J8" t="str">
+      <c r="J11" t="str">
         <v>Utang Usaha - Bahan Kimia</v>
       </c>
-      <c r="K8">
+      <c r="K11">
+        <v>125000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>21 Jan</v>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
+        <v>Voucher: Pembayaran Belanja Bahan Habis Pakai Tawas dll</v>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
+        <v>15.01.00</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Persediaan Bahan Kimia</v>
+      </c>
+      <c r="H12">
+        <v>125000</v>
+      </c>
+      <c r="I12" t="str">
+        <v>50.01.01</v>
+      </c>
+      <c r="J12" t="str">
+        <v>Utang Usaha - Bahan Kimia</v>
+      </c>
+      <c r="K12">
+        <v>125000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>21 Jan</v>
+      </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13" t="str">
+        <v>Voucher: Pembayaran Belanja Bahan Habis Pakai Tawas dll</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v>15.01.00</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Persediaan Bahan Kimia</v>
+      </c>
+      <c r="H13">
+        <v>125000</v>
+      </c>
+      <c r="I13" t="str">
+        <v>50.01.01</v>
+      </c>
+      <c r="J13" t="str">
+        <v>Utang Usaha - Bahan Kimia</v>
+      </c>
+      <c r="K13">
+        <v>125000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>21 Jan</v>
+      </c>
+      <c r="B14" t="str">
+        <v/>
+      </c>
+      <c r="C14" t="str">
+        <v>Voucher: Pembayaran Belanja Bahan Habis Pakai Tawas dll</v>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="str">
+        <v>15.01.00</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Persediaan Bahan Kimia</v>
+      </c>
+      <c r="H14">
+        <v>125000</v>
+      </c>
+      <c r="I14" t="str">
+        <v>50.01.01</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Utang Usaha - Bahan Kimia</v>
+      </c>
+      <c r="K14">
         <v>125000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>